<commit_message>
loads of improvements and updated results
</commit_message>
<xml_diff>
--- a/Results/2_parametrization/diagnostics/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
+++ b/Results/2_parametrization/diagnostics/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
@@ -11,13 +11,14 @@
     <sheet name="Computational_Time" sheetId="2" r:id="rId2"/>
     <sheet name="Final_Errors" sheetId="3" r:id="rId3"/>
     <sheet name="translational_sector" sheetId="4" r:id="rId4"/>
+    <sheet name="reaction_weights" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="31">
   <si>
     <t>run_id</t>
   </si>
@@ -49,6 +50,12 @@
     <t>E5</t>
   </si>
   <si>
+    <t>E4</t>
+  </si>
+  <si>
+    <t>E6</t>
+  </si>
+  <si>
     <t>f</t>
   </si>
   <si>
@@ -67,6 +74,12 @@
     <t>CE_R5_E5</t>
   </si>
   <si>
+    <t>CE_R4_E4</t>
+  </si>
+  <si>
+    <t>CE_R6_E6</t>
+  </si>
+  <si>
     <t>time_s</t>
   </si>
   <si>
@@ -86,6 +99,18 @@
   </si>
   <si>
     <t>R1</t>
+  </si>
+  <si>
+    <t>reaction</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>EX_ac_e</t>
+  </si>
+  <si>
+    <t>BIOMASS_Ec_iML1515_core_75p37M</t>
   </si>
 </sst>
 </file>
@@ -443,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -474,10 +499,10 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E2">
         <v>277.7777777777778</v>
@@ -494,13 +519,13 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E3">
-        <v>277.7777777777778</v>
+        <v>635.7718768659746</v>
       </c>
       <c r="F3">
         <v>0.9999999999643769</v>
@@ -514,13 +539,13 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E4">
-        <v>138.8888888888889</v>
+        <v>362.7161621880247</v>
       </c>
       <c r="F4">
         <v>0.9999999999643769</v>
@@ -534,13 +559,13 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E5">
-        <v>138.8888888888889</v>
+        <v>132.659306168434</v>
       </c>
       <c r="F5">
         <v>0.9999999999643769</v>
@@ -554,10 +579,10 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E6">
         <v>277.7777777777778</v>
@@ -574,13 +599,13 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E7">
-        <v>277.7777777777778</v>
+        <v>500.3424316953925</v>
       </c>
       <c r="F7">
         <v>0.9999999999643769</v>
@@ -594,16 +619,16 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E8">
-        <v>224.4506802599697</v>
+        <v>277.7777777777778</v>
       </c>
       <c r="F8">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -614,16 +639,16 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E9">
-        <v>1344.212742165005</v>
+        <v>277.7777777777778</v>
       </c>
       <c r="F9">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -634,16 +659,16 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E10">
-        <v>72.04001603913042</v>
+        <v>165.8826875569326</v>
       </c>
       <c r="F10">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -654,16 +679,16 @@
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E11">
-        <v>169.2295075395241</v>
+        <v>2540.349655517761</v>
       </c>
       <c r="F11">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -674,16 +699,16 @@
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E12">
-        <v>196.5183035825239</v>
+        <v>63.45673038798946</v>
       </c>
       <c r="F12">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -694,16 +719,16 @@
         <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E13">
-        <v>101.0028061169864</v>
+        <v>125</v>
       </c>
       <c r="F13">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -714,16 +739,16 @@
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E14">
-        <v>4313.733947807922</v>
+        <v>996.3928464550579</v>
       </c>
       <c r="F14">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -734,16 +759,16 @@
         <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E15">
-        <v>438.8184365148216</v>
+        <v>1492.469798872517</v>
       </c>
       <c r="F15">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -754,16 +779,16 @@
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E16">
-        <v>101.0028061169864</v>
+        <v>471.4085648766002</v>
       </c>
       <c r="F16">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -774,16 +799,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D17" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E17">
-        <v>4313.733947807922</v>
+        <v>943.9579413343153</v>
       </c>
       <c r="F17">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -794,16 +819,16 @@
         <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D18" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E18">
-        <v>661.7135472670827</v>
+        <v>19203.11819278318</v>
       </c>
       <c r="F18">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -814,16 +839,16 @@
         <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D19" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E19">
-        <v>101.0028061169864</v>
+        <v>1685.264015609272</v>
       </c>
       <c r="F19">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778475</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -834,16 +859,16 @@
         <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D20" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E20">
         <v>277.7777777777778</v>
       </c>
       <c r="F20">
-        <v>0.5943036166660929</v>
+        <v>0.6461873496247414</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -854,16 +879,16 @@
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D21" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21">
         <v>277.7777777777778</v>
       </c>
       <c r="F21">
-        <v>0.5943036166660929</v>
+        <v>0.6461873496247414</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -874,16 +899,16 @@
         <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D22" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E22">
-        <v>138.8888888888889</v>
+        <v>70.03649464928924</v>
       </c>
       <c r="F22">
-        <v>0.5943036166660929</v>
+        <v>0.6461873496247414</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -894,16 +919,16 @@
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D23" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E23">
-        <v>143.6068322991171</v>
+        <v>97.96373675618578</v>
       </c>
       <c r="F23">
-        <v>0.5943036166660929</v>
+        <v>0.6461873496247414</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -914,16 +939,16 @@
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E24">
-        <v>83.067886847425</v>
+        <v>267.2890637764092</v>
       </c>
       <c r="F24">
-        <v>0.5943036166660929</v>
+        <v>0.6461873496247414</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -934,16 +959,16 @@
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E25">
-        <v>125</v>
+        <v>265.3058069837629</v>
       </c>
       <c r="F25">
-        <v>0.5943036166660929</v>
+        <v>0.6461873496247414</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -954,16 +979,16 @@
         <v>6</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E26">
-        <v>714.5259311273028</v>
+        <v>228.1705168575217</v>
       </c>
       <c r="F26">
-        <v>0.6617064535818709</v>
+        <v>0.5851087708152268</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -974,16 +999,16 @@
         <v>7</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D27" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E27">
-        <v>262.5268882505852</v>
+        <v>459.6598049036785</v>
       </c>
       <c r="F27">
-        <v>0.6617064535818709</v>
+        <v>0.5851087708152268</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -994,16 +1019,16 @@
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D28" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E28">
-        <v>534.3971333669306</v>
+        <v>382.9195899432951</v>
       </c>
       <c r="F28">
-        <v>0.6617064535818709</v>
+        <v>0.5851087708152268</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1014,16 +1039,16 @@
         <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D29" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E29">
-        <v>680.1884930932147</v>
+        <v>671.2614414700107</v>
       </c>
       <c r="F29">
-        <v>0.6617064535818709</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1034,16 +1059,16 @@
         <v>7</v>
       </c>
       <c r="C30" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D30" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E30">
-        <v>1122.348932102825</v>
+        <v>975.6033238237552</v>
       </c>
       <c r="F30">
-        <v>0.6617064535818709</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1051,319 +1076,679 @@
         <v>2</v>
       </c>
       <c r="B31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C31" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E31">
-        <v>534.3971333669307</v>
+        <v>277.7777777777778</v>
       </c>
       <c r="F31">
-        <v>0.6617064535818709</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B32" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D32" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E32">
-        <v>1121.90316879916</v>
+        <v>277.7777777777778</v>
       </c>
       <c r="F32">
-        <v>0.6617064535818709</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B33" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E33">
-        <v>1124.445348971228</v>
+        <v>166.8583398272654</v>
       </c>
       <c r="F33">
-        <v>0.6617064535818709</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D34" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E34">
-        <v>534.3971333669308</v>
+        <v>91.26951679562232</v>
       </c>
       <c r="F34">
-        <v>0.6617064535818709</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E35">
-        <v>263.93581764026</v>
+        <v>1796.713251610602</v>
       </c>
       <c r="F35">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E36">
-        <v>845.5473511385883</v>
+        <v>416.6666666666667</v>
       </c>
       <c r="F36">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C37" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E37">
-        <v>92.29765205269445</v>
+        <v>268.2629196008958</v>
       </c>
       <c r="F37">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D38" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E38">
-        <v>138.8888888888889</v>
+        <v>432.178929850202</v>
       </c>
       <c r="F38">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C39" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D39" t="s">
         <v>15</v>
       </c>
       <c r="E39">
-        <v>125</v>
+        <v>975.6033238237552</v>
       </c>
       <c r="F39">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B40" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D40" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>1000.376070808028</v>
+        <v>3584.29944052269</v>
       </c>
       <c r="F40">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B41" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D41" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E41">
-        <v>845.5473511385883</v>
+        <v>91.26951679562235</v>
       </c>
       <c r="F41">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="42" spans="1:6">
       <c r="A42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D42" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E42">
-        <v>143.6068322991171</v>
+        <v>1036.609585830535</v>
       </c>
       <c r="F42">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="43" spans="1:6">
       <c r="A43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D43" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E43">
-        <v>1000.376070808028</v>
+        <v>322.2857188931086</v>
       </c>
       <c r="F43">
-        <v>0.6647462176800405</v>
+        <v>0.5851228207249695</v>
       </c>
     </row>
     <row r="44" spans="1:6">
       <c r="A44">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B44" t="s">
         <v>6</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D44" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E44">
-        <v>845.5473511385883</v>
+        <v>1850.949975302448</v>
       </c>
       <c r="F44">
-        <v>0.6647462176800405</v>
+        <v>0.5590747652536368</v>
       </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B45" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C45" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D45" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>143.6068322991171</v>
+        <v>381.6144618928222</v>
       </c>
       <c r="F45">
-        <v>0.6647462176800405</v>
+        <v>0.5590747652536368</v>
       </c>
     </row>
     <row r="46" spans="1:6">
       <c r="A46">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B46" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C46" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D46" t="s">
         <v>15</v>
       </c>
       <c r="E46">
-        <v>1000.376070808028</v>
+        <v>89.42097320029858</v>
       </c>
       <c r="F46">
-        <v>0.6647462176800405</v>
+        <v>0.5590747652536368</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47">
+        <v>1</v>
+      </c>
+      <c r="B47" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47">
+        <v>1231.525811453323</v>
+      </c>
+      <c r="F47">
+        <v>0.5590747652536368</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48">
+        <v>1</v>
+      </c>
+      <c r="B48" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" t="s">
+        <v>12</v>
+      </c>
+      <c r="D48" t="s">
+        <v>17</v>
+      </c>
+      <c r="E48">
+        <v>70.67438111070622</v>
+      </c>
+      <c r="F48">
+        <v>0.5590747652536368</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49">
+        <v>1</v>
+      </c>
+      <c r="B49" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" t="s">
+        <v>17</v>
+      </c>
+      <c r="E49">
+        <v>197.3530647956881</v>
+      </c>
+      <c r="F49">
+        <v>0.5590747652536368</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50">
+        <v>2</v>
+      </c>
+      <c r="B50" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" t="s">
+        <v>14</v>
+      </c>
+      <c r="E50">
+        <v>381.6144618928222</v>
+      </c>
+      <c r="F50">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51">
+        <v>2</v>
+      </c>
+      <c r="B51" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E51">
+        <v>943.3896139199124</v>
+      </c>
+      <c r="F51">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52">
+        <v>2</v>
+      </c>
+      <c r="B52" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" t="s">
+        <v>12</v>
+      </c>
+      <c r="D52" t="s">
+        <v>16</v>
+      </c>
+      <c r="E52">
+        <v>5454.388104782212</v>
+      </c>
+      <c r="F52">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53">
+        <v>2</v>
+      </c>
+      <c r="B53" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" t="s">
+        <v>16</v>
+      </c>
+      <c r="E53">
+        <v>160.2632511988367</v>
+      </c>
+      <c r="F53">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54">
+        <v>2</v>
+      </c>
+      <c r="B54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" t="s">
+        <v>12</v>
+      </c>
+      <c r="D54" t="s">
+        <v>18</v>
+      </c>
+      <c r="E54">
+        <v>78.80171365623809</v>
+      </c>
+      <c r="F54">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55">
+        <v>2</v>
+      </c>
+      <c r="B55" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" t="s">
+        <v>18</v>
+      </c>
+      <c r="E55">
+        <v>78.52709012300693</v>
+      </c>
+      <c r="F55">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56">
+        <v>2</v>
+      </c>
+      <c r="B56" t="s">
+        <v>9</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" t="s">
+        <v>17</v>
+      </c>
+      <c r="E56">
+        <v>204.0013955635647</v>
+      </c>
+      <c r="F56">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>11</v>
+      </c>
+      <c r="C57" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57" t="s">
+        <v>19</v>
+      </c>
+      <c r="E57">
+        <v>416.6666666666667</v>
+      </c>
+      <c r="F57">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58">
+        <v>2</v>
+      </c>
+      <c r="B58" t="s">
+        <v>11</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" t="s">
+        <v>19</v>
+      </c>
+      <c r="E58">
+        <v>786.0899423997445</v>
+      </c>
+      <c r="F58">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59">
+        <v>3</v>
+      </c>
+      <c r="B59" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" t="s">
+        <v>14</v>
+      </c>
+      <c r="E59">
+        <v>381.6144618928222</v>
+      </c>
+      <c r="F59">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60">
+        <v>3</v>
+      </c>
+      <c r="B60" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" t="s">
+        <v>15</v>
+      </c>
+      <c r="E60">
+        <v>943.3896139199124</v>
+      </c>
+      <c r="F60">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61">
+        <v>3</v>
+      </c>
+      <c r="B61" t="s">
+        <v>8</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" t="s">
+        <v>16</v>
+      </c>
+      <c r="E61">
+        <v>160.2632511988367</v>
+      </c>
+      <c r="F61">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62">
+        <v>3</v>
+      </c>
+      <c r="B62" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62" t="s">
+        <v>18</v>
+      </c>
+      <c r="E62">
+        <v>78.52709012300694</v>
+      </c>
+      <c r="F62">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63">
+        <v>3</v>
+      </c>
+      <c r="B63" t="s">
+        <v>9</v>
+      </c>
+      <c r="C63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" t="s">
+        <v>17</v>
+      </c>
+      <c r="E63">
+        <v>204.0013955635647</v>
+      </c>
+      <c r="F63">
+        <v>0.9968697152364935</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64">
+        <v>3</v>
+      </c>
+      <c r="B64" t="s">
+        <v>11</v>
+      </c>
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>19</v>
+      </c>
+      <c r="E64">
+        <v>786.0899423997442</v>
+      </c>
+      <c r="F64">
+        <v>0.9968697152364935</v>
       </c>
     </row>
   </sheetData>
@@ -1381,10 +1766,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1392,10 +1777,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.9842005519985833</v>
+        <v>0.9895101820000036</v>
       </c>
       <c r="C2">
-        <v>0.0002733890422218287</v>
+        <v>0.0002748639394444454</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1403,10 +1788,10 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2.288343125999745</v>
+        <v>2.942375764999952</v>
       </c>
       <c r="C3">
-        <v>0.0006356508683332626</v>
+        <v>0.0008173266013888754</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1414,10 +1799,10 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2.004759779001688</v>
+        <v>2.045979589999888</v>
       </c>
       <c r="C4">
-        <v>0.0005568777163893578</v>
+        <v>0.0005683276638888578</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1425,10 +1810,10 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1.941798604000724</v>
+        <v>2.061940100999891</v>
       </c>
       <c r="C5">
-        <v>0.0005393885011113121</v>
+        <v>0.0005727611391666364</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1436,10 +1821,10 @@
         <v>0</v>
       </c>
       <c r="B6">
-        <v>9.493006474998765</v>
+        <v>8.95824311299998</v>
       </c>
       <c r="C6">
-        <v>0.002636946243055212</v>
+        <v>0.002488400864722217</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1447,10 +1832,10 @@
         <v>1</v>
       </c>
       <c r="B7">
-        <v>2.38835925300009</v>
+        <v>2.384963512000013</v>
       </c>
       <c r="C7">
-        <v>0.0006634331258333582</v>
+        <v>0.000662489864444448</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1458,10 +1843,10 @@
         <v>2</v>
       </c>
       <c r="B8">
-        <v>2.063558162000845</v>
+        <v>13.40863167600014</v>
       </c>
       <c r="C8">
-        <v>0.0005732106005557903</v>
+        <v>0.003724619910000039</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1469,10 +1854,10 @@
         <v>3</v>
       </c>
       <c r="B9">
-        <v>1.907102728999234</v>
+        <v>2.097704186999863</v>
       </c>
       <c r="C9">
-        <v>0.0005297507580553428</v>
+        <v>0.0005826956074999619</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1480,10 +1865,10 @@
         <v>1</v>
       </c>
       <c r="B10">
-        <v>2.504229678001138</v>
+        <v>3.148092240999858</v>
       </c>
       <c r="C10">
-        <v>0.0006956193550003162</v>
+        <v>0.0008744700669444051</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1491,10 +1876,10 @@
         <v>2</v>
       </c>
       <c r="B11">
-        <v>1.940367987999707</v>
+        <v>5.315431563999937</v>
       </c>
       <c r="C11">
-        <v>0.0005389911077776964</v>
+        <v>0.00147650876777776</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1502,10 +1887,10 @@
         <v>3</v>
       </c>
       <c r="B12">
-        <v>1.964287032000357</v>
+        <v>2.511884722000104</v>
       </c>
       <c r="C12">
-        <v>0.0005456352866667658</v>
+        <v>0.0006977457561111401</v>
       </c>
     </row>
   </sheetData>
@@ -1523,7 +1908,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1539,7 +1924,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778474</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1547,7 +1932,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778474</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1555,7 +1940,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.5781610934725928</v>
+        <v>0.6439504786778474</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1563,7 +1948,7 @@
         <v>0</v>
       </c>
       <c r="B6">
-        <v>0.5943036166660929</v>
+        <v>0.6461873496247414</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1571,7 +1956,7 @@
         <v>1</v>
       </c>
       <c r="B7">
-        <v>0.6617064535818709</v>
+        <v>0.5851087708368838</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1579,7 +1964,7 @@
         <v>2</v>
       </c>
       <c r="B8">
-        <v>0.6617064535818709</v>
+        <v>0.5851228207466265</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1587,7 +1972,7 @@
         <v>3</v>
       </c>
       <c r="B9">
-        <v>0.6617064535818709</v>
+        <v>0.5851228207466265</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1595,7 +1980,7 @@
         <v>1</v>
       </c>
       <c r="B10">
-        <v>0.6647462176800405</v>
+        <v>0.5590747652536368</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1603,7 +1988,7 @@
         <v>2</v>
       </c>
       <c r="B11">
-        <v>0.6647462176800405</v>
+        <v>0.9968697152463304</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1611,7 +1996,7 @@
         <v>3</v>
       </c>
       <c r="B12">
-        <v>0.6647462176800405</v>
+        <v>0.9968697152463304</v>
       </c>
     </row>
   </sheetData>
@@ -1626,24 +2011,58 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B2">
         <v>1E-05</v>
       </c>
       <c r="C2">
         <v>1E-05</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>